<commit_message>
Update economic data 2026-10-05
</commit_message>
<xml_diff>
--- a/data/長期系列_CI指数_DI指数_DI景気指標.xlsx
+++ b/data/長期系列_CI指数_DI指数_DI景気指標.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="O:\CI\０１／CI\０１／速報\★R8(2026)★\令和8年7月分\g研究所ホームページ掲載宛送付ファイル\jp\stat\di\di\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="O:\CI\０１／CI\０２／速報からの改訂\★R8(2026)★\令和8年7月改訂\g研究所ホームページ掲載宛送付ファイル\jp\stat\di\di\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{FAB3867F-20A6-4532-A136-412B70E310B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{729D4610-6BD2-43A5-B3C1-EFEC4774FC9F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3240" yWindow="3240" windowWidth="17280" windowHeight="8880" xr2:uid="{20C0A5A3-949E-4EFC-A5B2-8DEDB94C117F}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{D4185C6C-2ACF-4442-85B9-415D9FE3133A}"/>
   </bookViews>
   <sheets>
     <sheet name="指数 Indexes" sheetId="1" r:id="rId1"/>
@@ -2454,7 +2454,7 @@
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="標準" xfId="0" builtinId="0"/>
-    <cellStyle name="標準 2" xfId="1" xr:uid="{2A7B69C9-16E4-44D7-ABDC-B8084B641E75}"/>
+    <cellStyle name="標準 2" xfId="1" xr:uid="{D1EEFFCF-E3D1-4C1D-A6BB-44A8B72E9776}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -2823,7 +2823,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AFD838BA-7B18-42E1-B44D-F1562AA0BF3D}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{02E850F8-4A33-4528-BCB0-CBC0EE2C6D66}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
@@ -28457,7 +28457,7 @@
         <v>118.3</v>
       </c>
       <c r="F562" s="4">
-        <v>111.7</v>
+        <v>111.6</v>
       </c>
       <c r="G562" s="4">
         <v>113.6</v>
@@ -28466,7 +28466,7 @@
         <v>116</v>
       </c>
       <c r="I562" s="4">
-        <v>108.4</v>
+        <v>108.3</v>
       </c>
       <c r="J562" s="4">
         <v>54.5</v>
@@ -28504,7 +28504,7 @@
         <v>118.3</v>
       </c>
       <c r="F563" s="4">
-        <v>111.3</v>
+        <v>111.2</v>
       </c>
       <c r="G563" s="4">
         <v>113.9</v>
@@ -28551,7 +28551,7 @@
         <v>118.9</v>
       </c>
       <c r="F564" s="4">
-        <v>111.7</v>
+        <v>111.8</v>
       </c>
       <c r="G564" s="4">
         <v>113.8</v>
@@ -28560,7 +28560,7 @@
         <v>116.5</v>
       </c>
       <c r="I564" s="4">
-        <v>108.4</v>
+        <v>108.5</v>
       </c>
       <c r="J564" s="4">
         <v>54.5</v>
@@ -28569,7 +28569,7 @@
         <v>75</v>
       </c>
       <c r="L564" s="4">
-        <v>33.299999999999997</v>
+        <v>44.4</v>
       </c>
       <c r="M564" s="4">
         <v>1385.5</v>
@@ -28578,7 +28578,7 @@
         <v>3265</v>
       </c>
       <c r="O564" s="4">
-        <v>3073.7</v>
+        <v>3084.8</v>
       </c>
     </row>
     <row r="565" spans="1:15" x14ac:dyDescent="0.2">
@@ -28592,40 +28592,40 @@
         <v>7</v>
       </c>
       <c r="D565" s="4">
-        <v>117.9</v>
+        <v>117.7</v>
       </c>
       <c r="E565" s="4">
         <v>120.6</v>
       </c>
       <c r="F565" s="4">
-        <v>113.3</v>
+        <v>113</v>
       </c>
       <c r="G565" s="4">
-        <v>115.5</v>
+        <v>115.2</v>
       </c>
       <c r="H565" s="4">
-        <v>118.1</v>
+        <v>118.2</v>
       </c>
       <c r="I565" s="4">
-        <v>109.9</v>
+        <v>109.6</v>
       </c>
       <c r="J565" s="4">
-        <v>66.7</v>
+        <v>65</v>
       </c>
       <c r="K565" s="4">
-        <v>93.8</v>
+        <v>94.4</v>
       </c>
       <c r="L565" s="4">
-        <v>75</v>
+        <v>62.5</v>
       </c>
       <c r="M565" s="4">
-        <v>1402.2</v>
+        <v>1400.5</v>
       </c>
       <c r="N565" s="4">
-        <v>3308.8</v>
+        <v>3309.4</v>
       </c>
       <c r="O565" s="4">
-        <v>3098.7</v>
+        <v>3097.3</v>
       </c>
     </row>
     <row r="574" spans="1:15" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
Update economic data 2026-10-12
</commit_message>
<xml_diff>
--- a/data/長期系列_CI指数_DI指数_DI景気指標.xlsx
+++ b/data/長期系列_CI指数_DI指数_DI景気指標.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="O:\CI\０１／CI\０２／速報からの改訂\★R8(2026)★\令和8年7月改訂\g研究所ホームページ掲載宛送付ファイル\jp\stat\di\di\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="O:\CI\０１／CI\０１／速報\★R8(2026)★\令和8年8月分\g研究所ホームページ掲載宛送付ファイル\jp\stat\di\di\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{729D4610-6BD2-43A5-B3C1-EFEC4774FC9F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{D7D1406F-068D-47A1-A940-6E502BAC390A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{D4185C6C-2ACF-4442-85B9-415D9FE3133A}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{152F49EE-67C0-4EAA-926D-5801C9071871}"/>
   </bookViews>
   <sheets>
     <sheet name="指数 Indexes" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="625" uniqueCount="583">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="626" uniqueCount="584">
   <si>
     <t>ＤＩ指数</t>
   </si>
@@ -2360,6 +2360,10 @@
   </si>
   <si>
     <t>2026000707</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>2026000808</t>
     <phoneticPr fontId="2"/>
   </si>
 </sst>
@@ -2454,7 +2458,7 @@
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="標準" xfId="0" builtinId="0"/>
-    <cellStyle name="標準 2" xfId="1" xr:uid="{D1EEFFCF-E3D1-4C1D-A6BB-44A8B72E9776}"/>
+    <cellStyle name="標準 2" xfId="1" xr:uid="{6FA56CAD-41B2-427F-8AF5-8ADFEDFE369A}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -2823,11 +2827,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{02E850F8-4A33-4528-BCB0-CBC0EE2C6D66}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A927F6A3-4DC9-4AA7-BA62-95C707730231}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:P574"/>
+  <dimension ref="A1:P575"/>
   <sheetFormatPr defaultRowHeight="13.2" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="11.6640625" bestFit="1" customWidth="1"/>
@@ -28263,7 +28267,7 @@
         <v>12</v>
       </c>
       <c r="D558" s="4">
-        <v>110.4</v>
+        <v>110.5</v>
       </c>
       <c r="E558" s="4">
         <v>114.6</v>
@@ -28413,7 +28417,7 @@
         <v>111.6</v>
       </c>
       <c r="G561" s="4">
-        <v>113.2</v>
+        <v>113.1</v>
       </c>
       <c r="H561" s="4">
         <v>114.7</v>
@@ -28554,7 +28558,7 @@
         <v>111.8</v>
       </c>
       <c r="G564" s="4">
-        <v>113.8</v>
+        <v>113.7</v>
       </c>
       <c r="H564" s="4">
         <v>116.5</v>
@@ -28592,7 +28596,7 @@
         <v>7</v>
       </c>
       <c r="D565" s="4">
-        <v>117.7</v>
+        <v>117.6</v>
       </c>
       <c r="E565" s="4">
         <v>120.6</v>
@@ -28610,7 +28614,7 @@
         <v>109.6</v>
       </c>
       <c r="J565" s="4">
-        <v>65</v>
+        <v>55</v>
       </c>
       <c r="K565" s="4">
         <v>94.4</v>
@@ -28619,7 +28623,7 @@
         <v>62.5</v>
       </c>
       <c r="M565" s="4">
-        <v>1400.5</v>
+        <v>1390.5</v>
       </c>
       <c r="N565" s="4">
         <v>3309.4</v>
@@ -28628,13 +28632,60 @@
         <v>3097.3</v>
       </c>
     </row>
-    <row r="574" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="D574" s="3"/>
-      <c r="E574" s="3"/>
-      <c r="F574" s="3"/>
-      <c r="G574" s="3"/>
-      <c r="H574" s="3"/>
-      <c r="I574" s="3"/>
+    <row r="566" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A566" s="13" t="s">
+        <v>583</v>
+      </c>
+      <c r="B566" s="2">
+        <v>2026</v>
+      </c>
+      <c r="C566" s="2">
+        <v>8</v>
+      </c>
+      <c r="D566" s="4">
+        <v>118</v>
+      </c>
+      <c r="E566" s="4">
+        <v>118.7</v>
+      </c>
+      <c r="F566" s="4">
+        <v>112.1</v>
+      </c>
+      <c r="G566" s="4">
+        <v>115.6</v>
+      </c>
+      <c r="H566" s="4">
+        <v>116.2</v>
+      </c>
+      <c r="I566" s="4">
+        <v>108.6</v>
+      </c>
+      <c r="J566" s="4">
+        <v>77.8</v>
+      </c>
+      <c r="K566" s="4">
+        <v>43.8</v>
+      </c>
+      <c r="L566" s="4">
+        <v>50</v>
+      </c>
+      <c r="M566" s="4">
+        <v>1418.3</v>
+      </c>
+      <c r="N566" s="4">
+        <v>3303.2</v>
+      </c>
+      <c r="O566" s="4">
+        <v>3097.3</v>
+      </c>
+    </row>
+    <row r="575" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="D575" s="3"/>
+      <c r="E575" s="3"/>
+      <c r="F575" s="3"/>
+      <c r="G575" s="3"/>
+      <c r="H575" s="3"/>
+      <c r="I575" s="3"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2"/>

</xml_diff>